<commit_message>
feat: add field validation and batch maintenance for knowledge libraries
</commit_message>
<xml_diff>
--- a/demo-knowledge-files/demo-abnormal-cases.xlsx
+++ b/demo-knowledge-files/demo-abnormal-cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="58">
   <si>
     <t>异常编号</t>
   </si>
@@ -130,7 +130,7 @@
     <t>压接参数</t>
   </si>
   <si>
-    <t>压接高度超上限 0.04 mm</t>
+    <t>压接高度超过上限 0.04 mm</t>
   </si>
   <si>
     <t>压接机微调后未同步首件记录</t>
@@ -149,6 +149,42 @@
   </si>
   <si>
     <t>压接高度,首件,拉力</t>
+  </si>
+  <si>
+    <t>V2.4 演示用待复核异常</t>
+  </si>
+  <si>
+    <t>ABN-HV-SEAL-MISSING</t>
+  </si>
+  <si>
+    <t>防水栓漏装导致外观复检不合格</t>
+  </si>
+  <si>
+    <t>后段 B1 预装工位</t>
+  </si>
+  <si>
+    <t>防水件装配</t>
+  </si>
+  <si>
+    <t>连接器背部缺少 1 个防水栓</t>
+  </si>
+  <si>
+    <t>换线后首件未逐孔点检</t>
+  </si>
+  <si>
+    <t>隔离批次并按孔位清单全检补装</t>
+  </si>
+  <si>
+    <t>预装首件必须拍照留痕</t>
+  </si>
+  <si>
+    <t>critical</t>
+  </si>
+  <si>
+    <t>防水栓,漏装,全检</t>
+  </si>
+  <si>
+    <t>V2.4 演示用 critical 异常</t>
   </si>
 </sst>
 </file>
@@ -535,7 +571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="17" width="16" customWidth="1"/>
@@ -697,7 +733,60 @@
         <v>45</v>
       </c>
       <c r="Q3" t="s">
-        <v>33</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J4" t="s">
+        <v>51</v>
+      </c>
+      <c r="K4" t="s">
+        <v>52</v>
+      </c>
+      <c r="L4" t="s">
+        <v>53</v>
+      </c>
+      <c r="M4" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>